<commit_message>
vault backup: 2026-08-02 17:09:20
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/Vibe lawyering/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/Vibe lawyering/anki/anki.xlsx
@@ -36,17 +36,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vibe lawyering</t>
+          <t>Alas</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Mr Rafique is far from alone in turning to AI rather than to costly lawyers--a trend professionals call "vibe lawyering". 译：Rafique 先生远不是唯一一个放弃昂贵律师、转而求助 AI 的人，法律专业人士把这一趋势称为“凭感觉打官司”。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：vibe = 氛围、感觉；lawyering = 做律师工作/处理法律事务；合起来指“凭 AI 给出的感觉来处理法律问题”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：科技新词 + 作者态度。它不是正式法律术语，带轻微讽刺，暗示行为缺少专业判断。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：vibe 原本是口语中的“感觉、氛围”，lawyering 是 lawyer 的动名词化，指从事法律工作。English: the phrase turns a casual word into a professional context, creating an ironic contrast between loose feeling and strict legal procedure.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：vibe 不只是“气氛”，在现代媒体中常指直觉式判断；lawyer 不只作名词，也可派生出 lawyering 表示法律操作。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：journalistic, ironic, mildly critical</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Alas for Mr Rafique, not only did he fail to submit the correct documents, but his filings were full of fake case law generated by an AI chatbot. 译：可惜的是，对 Rafique 先生来说，他不仅没有提交正确文件，而且他的诉讼材料里充满了由 AI 聊天机器人生成的虚假判例。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：唉；可惜；遗憾的是。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：外刊常用轻讽刺/转折信号词。它提示后文结果不利，常服务作者态度题。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：alas 是感叹副词，放句首时表示遗憾或讽刺。English: alas introduces an unfortunate outcome and often gives the sentence a lightly ironic tone.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：不是普通 but/however 的逻辑转折，而是带情绪色彩的“不幸的是”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：literary, ironic, mildly sympathetic</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章用该词概括普通人依赖 AI 起草法律文件、甚至编造判例的现象。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：诙谐点在于法律本应严谨，vibe 却很随意，形成反差。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：可能考标题含义、作者态度、科技便利与风险之间的转折。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到引号中的新词，要结合上下文判断定义和作者态度，不能只按字面翻译。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：rough AI-assisted legal work; careless self-help law / professional legal advice, verified legal service&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Vibe lawyering may save money at first, but it can fill court papers with unreliable claims. 译：凭感觉打官司起初可能省钱，却可能让诉讼文件充满不可靠主张。 2. The company avoided vibe lawyering and asked a qualified lawyer to review the contract. 译：这家公司没有凭感觉处理法律事务，而是请合格律师审查合同。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Technology should reduce barriers to public services, but vibe lawyering shows that convenience without verification can damage justice. 译：科技应降低公共服务门槛，但“凭感觉打官司”说明，缺乏核验的便利可能损害司法。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、社会责任、公共伦理、AI 与职业</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用 Alas 先给 Rafique 一点同情，再转入他的 AI 法律文件错误。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：有一点幽默和讽刺：当事人想借 AI 赢官司，结果因 AI 生成假判例败诉。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题、语气题、段落转折定位。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 Alas，后面通常是不利结果；选项若说作者完全赞同当事人，通常不稳。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：unfortunately, sadly, regrettably / fortunately, successfully&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Alas, the cheap legal template led the tenant to miss an important deadline. 译：可惜的是，廉价法律模板让租客错过了重要期限。 2. Alas, the school's new app saved time but exposed students' private data. 译：遗憾的是，学校的新应用节省了时间，却暴露了学生隐私。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Alas, convenience without responsibility can turn a useful technology into a public risk. 译：遗憾的是，缺乏责任的便利可能把有用技术变成公共风险。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技风险、公共责任、议论文转折</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -58,17 +58,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>trial and error</t>
+          <t>accuse A of doing B</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The article is titled "Trial and error" to connect court trials with the errors caused by AI use. 译：文章标题“试验与错误”把法庭审判和 AI 使用造成的错误联系起来。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：通过不断尝试和犯错来摸索；本文中 trial 还暗指“审判”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：标题双关。trial 既可指“试验”，也可指“审判”；error 指 AI 生成的法律错误。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：trial = 试验/审判，error = 错误。English: the idiom usually means learning by experiment, but the legal context activates the courtroom meaning of trial.&lt;br&gt;&lt;b&gt;多义项详解&lt;/b&gt;：trial: 1. 审判，如 a criminal trial；2. 试验，如 a clinical trial；3. 考验，如 a trial of patience。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：witty, ironic, headline-style</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：When Britain's tax authorities accused Omar Rafique of deliberately underpaying his restaurant's taxes, he challenged them in court. 译：当英国税务机关指控 Omar Rafique 故意少缴其餐馆税款时，他选择上法庭提出抗辩。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：指控 A 做了 B。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：法律/新闻高频搭配，of 后接名词或动名词；注意 accused 不等于 proved。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：accuse = 指控，A 是被指控对象，of doing B 是指控内容。English: accuse reports an allegation, not a confirmed fact.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：accuse sb of sth/doing sth；be accused of corruption/fraud/pollution。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, accusatory</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：标题预告文章会讨论法律 AI 的试错以及由此产生的司法错误。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：标题题、主旨题可能要求识别双关和全文核心风险。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：遇到标题中的普通词，要回到文章领域判断是否有双关。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Medical innovation often advances through trial and error, but patient safety must come first. 译：医学创新常常通过试错推进，但患者安全必须优先。 2. A start-up may learn by trial and error, but a court cannot accept invented evidence. 译：初创企业可以通过试错学习，但法院不能接受编造的证据。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Social progress may involve trial and error, but every experiment should be guided by responsibility. 译：社会进步可能包含试错，但每一次尝试都应由责任引导。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技创新、教育学习、公共治理</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：税务机关指控 Rafique 故意少缴税，这是案件开端。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：该表达只说明“被指控”，不说明事实已经成立，阅读中要区分 claim 和 fact。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题、事实与主张区分、翻译固定搭配。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：选项把 accuse 改成 prove/confirm 通常偷换；把 of doing 误译为目的也不对。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：charge A with doing B, allege that A did B / prove A did B&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Residents accused the factory of releasing untreated waste into the river. 译：居民指控工厂向河流排放未经处理的废水。 2. The company was accused of using customer data without clear consent. 译：该公司被指控在未获得明确同意的情况下使用客户数据。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public trust declines when powerful institutions are accused of hiding important information. 译：当强势机构被指控隐瞒重要信息时，公众信任会下降。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律新闻、环境保护、企业责任</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -80,17 +80,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tax authorities</t>
+          <t>underpay taxes / underpay workers</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：When Britain's tax authorities accused Omar Rafique of deliberately underpaying his restaurant's taxes, he challenged them in court. 译：当英国税务机关指控 Omar Rafique 故意少缴其餐馆税款时，他选择上法庭提出抗辩。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：税务机关；负责征税、审查税款和执法的官方机构。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：authorities 常指“官方机构/当局”，不是抽象的“权威”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：tax = 税，authorities = 当局/政府部门。English: authorities in news writing often means official bodies with legal power, not experts with knowledge.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：authority: 1. 权威；2. 权力；3. 当局。复数 authorities 高频译为“有关部门/当局”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, institutional, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Britain's tax authorities accused him of deliberately underpaying his restaurant's taxes. 译：英国税务机关指控他故意少缴其餐馆税款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：少缴税款；少付工资。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：under- 前缀高频表示“不足、低于应有水平”；经济/职场/社会责任话题可迁移。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：under- = too little/below the proper level；pay = 支付。English: underpay means to pay less than required, whether taxes, wages or bills.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：可指少缴税、少付工资；underestimate 低估，underfund 资金不足，underreport 少报。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：negative, economic/legal</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：税务机关是法律纠纷的起点，说明案件并非私人争吵，而是与公共执法有关。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节定位题可能把 tax authorities 改写为 tax officials 或 government agencies。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：tax officials, revenue agencies / tax experts, financial advisers&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Tax authorities investigated the company after its reported profits suddenly fell. 译：该公司申报利润突然下降后，税务机关展开调查。 2. Small businesses often need clear guidance from tax authorities. 译：小企业常常需要税务机关给出清晰指导。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Tax authorities should make rules transparent so that ordinary citizens can comply with them. 译：税务机关应让规则透明，以便普通公民遵守。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：经济生活、公共治理、法律阅读</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：原文中 underpay 指少缴税，且 deliberately 加重责任色彩。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：少缴税不只是财务问题，也涉及公共责任和公平负担。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词缀题、熟词构词、经济类细节题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 under- 先判断“不足/低于标准”，不要按“下面”直译。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：pay too little, evade part of tax / overpay, fully pay&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The restaurant underpaid taxes and gained an unfair advantage over honest competitors. 译：这家餐馆少缴税，从而相对守法竞争者获得不公平优势。 2. Employers who underpay workers weaken both dignity and productivity. 译：少付员工工资的雇主会削弱尊严和生产力。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：A responsible company should not underpay workers or taxes in pursuit of short-term profit. 译：负责任的公司不应为了短期利润少付工资或少缴税。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：经济伦理、职场公平、社会责任&lt;br&gt;&lt;b&gt;归一化合并&lt;/b&gt;：用户词表 underpay 归一化为 underpay taxes / underpay workers。</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -102,17 +102,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>deliberately underpay taxes</t>
+          <t>create a more level playing field</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Britain's tax authorities accused him of deliberately underpaying his restaurant's taxes. 译：英国税务机关指控他故意少缴其餐馆税款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：故意少缴税款。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：deliberately 是责任判断词，决定行为是失误还是故意。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：deliberate = 深思熟虑的/故意的，-ly 变副词；underpay = under- 少于 + pay 支付。English: under- often means too little or below the required level, as in underfund, underestimate, underreport.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：underpay 可指少付工资，也可指少缴税；deliberate 作形容词是“故意的”，作动词是“认真考虑”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：accusatory, legal, negative</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI "might create a more level playing field" for litigants representing themselves. 译：AI “或许能为自行出庭的诉讼当事人创造一个更公平的竞争环境”。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：创造一个更平坦的比赛场地；引申为让竞争更公平。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：比喻性短语，常用于教育公平、机会公平、科技普惠。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：level = 平的/公平的；playing field = 比赛场地。English: a level playing field means conditions in which no side has an unfair advantage.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：level 可作“水平”，也可作形容词“平坦的、公平的”；field 可指领域，也可指运动场。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：positive, policy-friendly, formal</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：这个指控让案件进入法庭，也强调 Rafique 面临的是严肃法律责任。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：完形和细节题会考 deliberately 与 accidentally/negligently 的区别。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 deliberately，要把作者/机构对行为性质的判断标出来。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The restaurant was fined because it deliberately underpaid taxes for several years. 译：这家餐馆因多年故意少缴税款而被罚。 2. An employer who deliberately underpays workers damages both trust and the labour market. 译：故意少付员工工资的雇主会损害信任和劳动力市场。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：A fair society cannot tolerate companies that deliberately underpay workers or taxes. 译：公平社会不能容忍故意少付工资或少缴税的企业。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：经济伦理、社会责任、职场公平</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：法官承认 AI 可能帮助没钱请律师的人，但这不等于法院会接受虚假材料。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题要识别让步：作者承认好处，但核心仍是风险。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：make access fairer, reduce inequality / guarantee success, remove all legal barriers&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Online courses can create a more level playing field for students in poor regions. 译：在线课程能为贫困地区学生创造更公平的竞争环境。 2. Transparent hiring rules create a more level playing field for young workers. 译：透明的招聘规则为年轻劳动者创造更公平的竞争环境。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public policy should create a more level playing field for people with fewer resources. 译：公共政策应为资源较少的人创造更公平的竞争环境。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育公平、就业公平、数字鸿沟、社会责任</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -124,17 +124,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>challenge someone in court</t>
+          <t>throw the case out</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：When Britain's tax authorities accused Omar Rafique of deliberately underpaying his restaurant's taxes, he challenged them in court. 译：当英国税务机关指控 Omar Rafique 故意少缴其餐馆税款时，他在法庭上提出抗辩。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在法庭上挑战/质疑某人的决定或指控。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：challenge 不是“挑战比赛”，而是“质疑、反对、提出异议”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：challenge + decision/claim/authority 表示对决定、主张或权力提出质疑。English: in legal and academic contexts, challenge means to question the validity of something.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：challenge: 1. 挑战；2. 质疑；3. 难题。本文取第 2 义。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, confrontational</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Though the judge noted AI's possible benefit, she threw the case out on May 6th. 译：尽管法官指出 AI 可能有益，她仍在 5 月 6 日驳回了该案。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：把案件扔出去；法律含义是“驳回案件”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语。out 常含“排除、淘汰、离开程序”的意思。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：throw out = 丢弃/拒绝/驳回；case = 案件。English: in legal reporting, throw out a case means dismiss it because it is procedurally or substantively defective.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：case 可指案件、情况、病例、论点；throw out 可指扔掉、驱逐、否决。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：journalistic, informal but accepted in legal reporting</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Rafique 没有接受税务指控，而是进入司法程序。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：challenge a policy/decision 常被同义替换为 dispute, contest, question。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Residents challenged the pollution permit in court after the factory expanded. 译：工厂扩建后，居民在法庭上质疑其排污许可。 2. The student challenged the university's decision in court and asked for a review. 译：这名学生在法庭上质疑学校决定，并要求复审。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Citizens should have lawful channels to challenge unfair decisions in court. 译：公民应有合法渠道在法庭上质疑不公决定。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：公共治理、教育公平、环境保护</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：法官认可 AI 的潜在公平作用，但虚假判例使案件无法继续。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读题可能问 outcome；选项中 dismiss/reject 是同义替换。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The court threw the case out because the evidence was unreliable. 译：法院因证据不可靠而驳回案件。 2. The judge may throw the case out if the plaintiff misses the deadline. 译：如果原告错过截止日期，法官可能驳回案件。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Rules should be clear enough that valid complaints are not thrown out for avoidable mistakes. 译：规则应足够清晰，以免有效投诉因可避免错误而被驳回。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律阅读、制度公平、程序正义</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -146,17 +146,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>filings were full of fake case law</t>
+          <t>AI hallucinations</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：His filings were full of fake case law generated by an AI chatbot. 译：他的诉讼材料里充满了由 AI 聊天机器人生成的虚假判例。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：提交文件里充满虚假判例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：filings 是法律/行政语境中的“提交文件”；case law 是“判例法/判例”，不能拆成“案件法律”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：file 作动词是“提交、归档”，filing 是提交的文件；fake = 虚假的；case law = 由法院判例形成的法律规则。English: legal filings are documents submitted to a court, and case law means precedent-based law.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：file: 文件/档案；提交；排成纵队。case: 案件/情况/箱子。law 在 case law 中指法律体系中的判例规则。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, critical, factual</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A top New York firm apologised to a court for errors caused by AI hallucinations. 译：一家纽约顶级律所因 AI 幻觉造成的错误向法院道歉。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：AI 的幻觉；指 AI 编造看似真实但并不存在的信息。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：科技类核心术语，可用于理解 AI 可靠性和信息核验。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：hallucination 本义是“幻觉”，AI hallucination 是比喻用法，指模型生成虚假内容。English: in AI, hallucination means fluent but false output, not a human medical symptom.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：hallucination 在医学中是“幻觉”，在 AI 中是“编造性输出”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：technical, cautionary, negative</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：这是案件失败的直接原因，说明 AI 不是只犯小错，而是制造法律依据错误。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题可能考 generated by... 后置定语；阅读题可能问法官驳回案件的原因。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：court documents, legal submissions, fabricated precedents / valid evidence, official tax forms&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The judge rejected the appeal because the filings were full of fake case law. 译：法官驳回上诉，因为提交材料中充满虚假判例。 2. A lawyer must verify every source before a filing is submitted to court. 译：律师在向法院提交文件前必须核验每一项来源。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Digital convenience becomes dangerous when public documents are full of fake case law or unchecked facts. 译：当公共文件充满虚假判例或未经核验的事实时，数字便利就会变得危险。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律科技、学术诚信、信息核验</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 幻觉导致律所向法院道歉，说明专业人士也不能免于风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能问 hallucinations 在科技语境中的含义，应选 fabricated output，而非 mental illness。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. AI hallucinations can produce confident answers with false statistics. 译：AI 幻觉可能生成带有虚假统计数据却语气自信的答案。 2. Doctors should not rely on AI hallucinations when making clinical decisions. 译：医生做临床决策时不应依赖 AI 编造内容。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI hallucinations remind us that speed is meaningless without accuracy. 译：AI 幻觉提醒我们，没有准确性，速度毫无意义。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、健康医疗、教育诚信</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -168,17 +168,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>generated by an AI chatbot</t>
+          <t>contractual dispute</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The fake case law was generated by an AI chatbot. 译：这些虚假判例是由 AI 聊天机器人生成的。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：由 AI 聊天机器人生成。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：过去分词短语作后置定语或被动结构，常用于科技文章说明来源。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：generate = 产生、生成；generated by... = 由……生成。English: generate often appears with data, text, energy, revenue and ideas; in AI contexts it means to produce output automatically.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：generate 不只表示“发电”，还表示“产生收入/生成文本/引发兴趣”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：technical, neutral, context-dependent</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Lawyers on both sides of a contractual dispute in Mississippi were fined for citing fabricated cases. 译：在密西西比州一起合同纠纷中，双方律师都因引用捏造案例而被罚款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：合同纠纷。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：contractual 是 contract 的形容词；dispute 是法律、国际关系、职场文章高频词。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：contract = 合同；-ual 形容词后缀；dispute = 争端/纠纷。English: contractual describes something arising from or governed by a contract.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：dispute 作名词是争端，作动词是质疑/争论；contract 作名词是合同，作动词可指收缩。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 生成内容被误当作法律依据，造成司法风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长难句中 `generated by...` 常修饰前面的名词，翻译时要前置为“由……生成的”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Reports generated by an AI chatbot should be checked before they are used in public decisions. 译：由 AI 聊天机器人生成的报告在用于公共决策前应被核查。 2. The image was generated by an AI chatbot, but the campaign team still reviewed its accuracy. 译：这张图片由 AI 聊天机器人生成，但宣传团队仍审查了其准确性。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Information generated by an AI chatbot should support human judgment, not replace it. 译：由 AI 聊天机器人生成的信息应支持人的判断，而不是取代人的判断。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、教育学习、信息素养</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：合同纠纷中的双方律师都引用捏造案例，说明 AI 错误影响专业法律实践。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中 dispute 可被替换为 conflict, disagreement, legal row。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The supplier and the factory entered a contractual dispute over delivery dates. 译：供应商和工厂因交货日期陷入合同纠纷。 2. Mediation can resolve a contractual dispute before it reaches court. 译：调解可以在合同纠纷进入法院前解决问题。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Clear rules can prevent a contractual dispute from damaging long-term cooperation. 译：清晰规则可以防止合同纠纷损害长期合作。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场商业、经济生活、法律阅读</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -190,17 +190,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>create a more level playing field</t>
+          <t>relying on AI can prove expensive</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI "might create a more level playing field" for litigants representing themselves. 译：AI “或许能为自行出庭的诉讼当事人创造一个更公平的竞争环境”。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：创造一个更平坦的比赛场地；引申为让竞争更公平。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：比喻性短语，常用于教育公平、机会公平、科技普惠。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：level = 平的/公平的；playing field = 比赛场地。English: a level playing field means conditions in which no side has an unfair advantage.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：level 可作“水平”，也可作形容词“平坦的、公平的”；field 可指领域，也可指运动场。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：positive, policy-friendly, formal</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：And relying on AI can prove expensive. 译：依赖 AI 也可能代价高昂。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：依赖 AI 可能最终证明很昂贵。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：prove + adj. = 结果证明是；expensive 可指金钱或代价。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：rely on = 依赖；prove expensive = 结果代价高昂。English: prove followed by an adjective describes the outcome, not the act of giving evidence.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：prove 不只表示“证明”，也可表示“结果是”；expensive 可引申为“造成严重后果”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：warning, concise, evaluative</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：法官承认 AI 可能帮助没钱请律师的人，但这不等于法院会接受虚假材料。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题要识别让步：作者承认好处，但核心仍是风险。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：make access fairer, reduce inequality / guarantee success, remove all legal barriers&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Online courses can create a more level playing field for students in poor regions. 译：在线课程能为贫困地区学生创造更公平的竞争环境。 2. Transparent hiring rules create a more level playing field for young workers. 译：透明的招聘规则为年轻劳动者创造更公平的竞争环境。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public policy should create a more level playing field for people with fewer resources. 译：公共政策应为资源较少的人创造更公平的竞争环境。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育公平、就业公平、数字鸿沟、社会责任</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：该句开启一组因 AI 使用不当而被罚款或道歉的例子。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题不要译成“证明昂贵”，应译为“结果可能代价高昂”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Relying on AI can prove expensive when legal facts are not checked. 译：如果不核查法律事实，依赖 AI 可能代价高昂。 2. Relying on cheap repairs can prove expensive when safety is ignored. 译：如果忽视安全，依赖廉价维修可能最终代价高昂。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Relying on AI can prove expensive when efficiency is pursued at the expense of responsibility. 译：当效率以牺牲责任为代价时，依赖 AI 可能代价高昂。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技依赖、健康建议、学习工具、职场效率</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -212,17 +212,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>litigants representing themselves</t>
+          <t>human lawyers still have their place</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The judge said AI might help litigants representing themselves. 译：法官说 AI 可能帮助自行代理的诉讼当事人。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：自己代表自己的诉讼当事人。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：represent 在法律语境中是“代理、代表”，不是“表现”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：litigant = 诉讼当事人，来自 litigate；represent oneself = 自行代理。English: a self-represented litigant appears in court without a lawyer.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：represent: 1. 代表；2. 象征；3. 代理；4. 表示。本文取法律代理义。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：For now, human lawyers still have their place. 译：至少目前，人类律师仍有其不可替代的位置。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：人类律师仍有自己的位置。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：have one's place = 仍有价值/仍有适用场景；用于平衡论证。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：place 不只是地点，也可指角色、位置、价值。English: to have one's place means to remain useful or appropriate within a changing system.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：place: 地方/位置/角色/社会地位。本文是“角色和价值”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：balanced, concluding, pragmatic</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章讨论的核心群体是没有律师、借助 AI 处理法律材料的人。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题可能把它改写为 people acting without lawyers。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Litigants representing themselves often struggle with deadlines and evidence rules. 译：自行代理的诉讼当事人常常难以处理截止日期和证据规则。 2. Courts provide guidance for litigants representing themselves, but they do not give legal advice. 译：法院会为自行代理的当事人提供指引，但不会提供法律建议。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public services should be designed so that citizens representing themselves are not excluded by complexity. 译：公共服务设计应避免让自行处理事务的公民因复杂程序而被排除在外。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律公平、公共服务、弱势群体支持</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章承认 AI 有用，但结论强调专业人类判断仍不可替代。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：主旨题和态度题可据此判断作者不是简单反 AI，而是主张谨慎分工。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Even in an age of online courses, human teachers still have their place. 译：即使在在线课程时代，人类教师仍有其价值。 2. Automated tools are useful, but human editors still have their place. 译：自动化工具很有用，但人类编辑仍有其位置。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：In the age of artificial intelligence, human judgment still has its place in education and public life. 译：在人工智能时代，人的判断在教育和公共生活中仍有其价值。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：AI 与职业、教育学习、医疗健康、文化传承</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -234,17 +234,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>throw the case out</t>
+          <t>represent oneself / represent themselves</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Though the judge noted AI's possible benefit, she threw the case out on May 6th. 译：尽管法官指出 AI 可能有益，她仍在 5 月 6 日驳回了该案。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：把案件扔出去；法律含义是“驳回案件”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语。out 常含“排除、淘汰、离开程序”的意思。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：throw out = 丢弃/拒绝/驳回；case = 案件。English: in legal reporting, throw out a case means dismiss it because it is procedurally or substantively defective.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：case 可指案件、情况、病例、论点；throw out 可指扔掉、驱逐、否决。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：journalistic, informal but accepted in legal reporting</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The judge noted that AI might create a more level playing field for litigants representing themselves. 译：法官指出，AI 可能为自行代理的诉讼当事人创造更公平的竞争环境。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：自行代理；自己代表自己。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：represent 的法律义是“代理/代表”，不是“表现”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：represent = 代表、代理；oneself/themselves 表示没有律师。English: to represent oneself is to act as one's own legal representative.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：represent 还可指“象征、体现”，如 represent social change。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：法官认可 AI 的潜在公平作用，但虚假判例使案件无法继续。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读题可能问 outcome；选项中 dismiss/reject 是同义替换。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The court threw the case out because the evidence was unreliable. 译：法院因证据不可靠而驳回案件。 2. The judge may throw the case out if the plaintiff misses the deadline. 译：如果原告错过截止日期，法官可能驳回案件。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Rules should be clear enough that valid complaints are not thrown out for avoidable mistakes. 译：规则应足够清晰，以免有效投诉因可避免错误而被驳回。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律阅读、制度公平、程序正义</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章核心群体是没请律师、借助 AI 自行处理案件的人。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：这个表达指向 access to justice：普通人进入法律系统的成本太高。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题、细节定位、长难句后置修饰。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：people acting without lawyers 是同义替换；不要译成“表现自己”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：self-representing litigants, act without lawyers / represented by lawyers&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Tenants who represent themselves often need clear instructions from the court. 译：自行代理的租客常需要法院提供清晰说明。 2. A student may represent herself in a disciplinary hearing if she cannot afford legal help. 译：如果请不起法律帮助，学生可能在纪律听证中自行代理。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public services should help citizens who represent themselves without lowering standards of evidence. 译：公共服务应帮助自行代理的公民，但不能降低证据标准。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律公平、公共服务、教育治理&lt;br&gt;&lt;b&gt;归一化合并&lt;/b&gt;：用户词表 representing themselves 与原候选 litigants representing themselves / self-representing litigants 合并。</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -256,17 +256,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>far from alone</t>
+          <t>far from alone in doing</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Mr Rafique is far from alone in turning to AI rather than to costly lawyers. 译：Rafique 先生远不是唯一一个放弃昂贵律师、转而求助 AI 的人。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：远非孤身一人；并不是个例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：从个案过渡到普遍趋势的高频句块。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：far from + adj./n. = 远非、完全不。English: far from intensifies negation; far from alone means many others do the same.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：far from 不表示物理距离，而表示否定程度。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, analytical, trend-signalling</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Mr Rafique is far from alone in turning to AI rather than to costly lawyers--a trend professionals call "vibe lawyering". 译：Rafique 先生远不是唯一一个放弃昂贵律师、转而求助 AI 的人，法律专业人士把这一趋势称为“凭感觉打官司”。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：远不是唯一做某事的人；并非个例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：个案转趋势的篇章信号，适合主旨题和段落功能题。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：far from = 远非，alone = 独自；in doing 说明具体行为。English: far from alone in doing something means many others are doing the same thing.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：far from 不表示空间距离，而是强烈否定。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：analytical, trend-signalling</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用该短语从 Rafique 个案转入“AI 代替律师”的整体趋势。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：篇章结构题中，它常是“个例 -&gt; 趋势”的信号。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The city is far from alone in facing a shortage of affordable housing. 译：这个城市绝不是唯一面临保障性住房短缺的城市。 2. Young workers are far from alone in using AI to draft routine emails. 译：年轻职场人并不是唯一用 AI 起草日常邮件的人。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：This problem is far from alone; it reflects a wider failure of public education. 译：这个问题并非个例；它反映了公共教育更广泛的不足。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：社会现象引入、教育问题、职场变化</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者从 Rafique 个案转入越来越多人用 AI 代替律师的社会趋势。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：它暗示问题不是个别倒霉案例，而是制度层面的新现象。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：段落功能题、主旨题、例证题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 far from alone，要往后找数据或更多例子来证明“趋势”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：not an isolated case, one of many / unique, exceptional&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The city is far from alone in struggling with housing costs. 译：这个城市并不是唯一被住房成本困扰的城市。 2. Young employees are far from alone in turning to AI for routine writing tasks. 译：年轻员工并不是唯一借助 AI 处理日常写作任务的人。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：This case is far from alone in showing how technology can expose institutional weaknesses. 译：这个案例并非个例，它说明科技会暴露制度弱点。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：社会现象、科技生活、职场变化</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -278,17 +278,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>turn to AI rather than costly lawyers</t>
+          <t>civil cases</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Many people are turning to AI rather than to costly lawyers. 译：许多人正在转向 AI，而不是求助昂贵的律师。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：转向 AI，而不是昂贵律师。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：turn to = 求助于/转向；rather than = 而不是，构成选择对比。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：turn to 强调在困难中寻找帮助；costly = 昂贵的/代价高的。English: turn to often collocates with experts, technology, government, family or old habits.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：costly 不只指价格高，也可指造成严重代价，如 costly mistakes。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：neutral but hints at economic pressure</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In England and Wales the share of civil cases in county courts with lawyers on both sides fell from 51% in 2022 to 42% last year. 译：在英格兰和威尔士，郡法院民事案件中双方都有律师代理的比例从 2022 年的 51% 降到了去年的 42%。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：民事案件。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：civil 在法律中是“民事的”，不是“文明的/市民的”；与 criminal cases 区分。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：civil = 民事的/公民的/文明的；case = 案件。English: civil cases involve disputes between people or organisations, not criminal prosecution by the state.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：civil: 民事的、公民的、文明的；case: 案件、情况、病例、论点。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：律师费用高是普通人依赖 AI 的重要背景。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：原因题可能把该短语改写为 seek help from AI because lawyers are expensive。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Small firms turn to AI rather than costly consultants when budgets are tight. 译：预算紧张时，小公司会转向 AI，而不是昂贵的咨询顾问。 2. Some patients turn to online advice rather than costly clinics, which can be risky. 译：一些患者转向网上建议而不是昂贵诊所，这可能有风险。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：People may turn to AI rather than costly services, so society must improve both access and reliability. 译：人们可能转向 AI 而不是昂贵服务，因此社会必须同时提高可及性和可靠性。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：经济生活、健康服务、教育资源、AI 普惠</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：原文用 civil cases 展示律师参与比例下降，说明自行代理正在增加。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：民事案件门槛相对低，更容易成为 AI 自助法律工具进入的场景。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题、法律类别区分、熟词僻义。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 civil + court/case/law，优先译为“民事”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：non-criminal cases, private disputes / criminal cases&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Civil cases often involve contracts, housing or employment disputes. 译：民事案件常涉及合同、住房或就业纠纷。 2. Online tools may help people prepare documents for simple civil cases. 译：在线工具可能帮助人们为简单民事案件准备文件。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Simpler procedures in civil cases can improve access to justice for ordinary citizens. 译：民事案件中更简单的程序可以改善普通公民获得司法救济的机会。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律阅读、社会公平、职场纠纷</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -300,17 +300,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>represent oneself in court</t>
+          <t>complaint</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In American federal civil courts 17% of people represented themselves in 2025. 译：在美国联邦民事法院，2025 年有 17% 的人自行代理自己出庭。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在法庭上代表自己。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：represent 的法律义；self-representation 与 access to justice 相关。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：represent = 代表/代理；oneself 表示没有外部代理人。English: to represent oneself is to act as one's own legal representative.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：represent 还可指“体现、象征”，如 represent social change。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They also find that this year 18% of complaints have probably contained AI-generated text. 译：他们还发现，今年 18% 的起诉状很可能包含 AI 生成文本。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：抱怨；投诉；法律中的起诉状。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词僻义。本文 complaint 不是普通“抱怨”，而是提交给法院的法律文件。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：complain = 抱怨/投诉；complaint = 抱怨、投诉，也可指起诉状。English: in legal contexts, a complaint is the document that starts a lawsuit.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：1. 日常抱怨；2. 消费投诉；3. 法律起诉状。本文取第 3 义。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal in legal context, neutral</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：自行代理比例上升为 vibe lawyering 提供了数据背景。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题常考比例变化和原因；翻译题注意不要译成“表现自己”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. A tenant may represent herself in court when she cannot afford a lawyer. 译：当租客请不起律师时，她可能在法庭上自行代理。 2. People who represent themselves in court need plain-language instructions. 译：在法庭上自行代理的人需要通俗清晰的说明。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：A fair legal system should help citizens who represent themselves in court understand basic procedures. 译：公平的法律体系应帮助在法庭上自行代理的公民理解基本程序。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：社会公平、公共服务、法律援助</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：研究发现相当比例的法律 complaint 可能包含 AI 生成文本。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：基础词进入法律语境后含义升级，是考研阅读常见陷阱。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题、翻译题、法律语境识别。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：complaint 与 court/lawsuit/filed 搭配时，优先考虑“起诉状”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：legal filing, lawsuit document / casual complaint&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The complaint contained several claims about unfair dismissal. 译：这份起诉状包含数项关于不公平解雇的主张。 2. The consumer filed a complaint after the company refused a refund. 译：公司拒绝退款后，消费者提出投诉。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Institutions should respond to a complaint with fairness rather than delay. 译：机构应公平回应投诉，而不是拖延。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律、消费者保护、职场公平</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -322,17 +322,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AI-generated text</t>
+          <t>contain AI-generated text</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They also find that this year 18% of complaints have probably contained AI-generated text. 译：他们还发现，今年 18% 的起诉状很可能包含 AI 生成文本。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：由 AI 生成的文本。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：复合形容词 + 过去分词；科技文章核心表达。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：AI-generated = AI 生成的；generated 是过去分词作定语。English: hyphenated modifiers like AI-generated, state-owned and evidence-based compress information before a noun.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：complaint 在法律中可指“起诉状”，不只是“抱怨”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：technical, neutral; risk depends on context</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：They also find that this year 18% of complaints have probably contained AI-generated text. 译：他们还发现，今年 18% 的起诉状很可能包含 AI 生成文本。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：包含 AI 生成文本。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：contain 是基础词，但在抽象名词搭配中常译为“包含、含有”，不译成“控制”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：contain = 包含/容纳/控制。English: contain can mean include something inside, or control the spread of something harmful.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：1. 包含，如 contain evidence；2. 容纳，如 contain 1,000 people；3. 控制，如 contain inflation/a virus。本文是“包含”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：neutral, factual</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：数据说明 AI 已经进入正式法律文件。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中 complaint 可能误导为普通“投诉”；这里是法律文件。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. AI-generated text can improve efficiency, but it must be reviewed before publication. 译：AI 生成文本可以提高效率，但发布前必须审核。 2. Schools need policies for AI-generated text in essays and reports. 译：学校需要针对论文和报告中的 AI 生成文本制定政策。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI-generated text should be treated as a draft, not as verified knowledge. 译：AI 生成文本应被视为草稿，而不是已核实的知识。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育诚信、科技生活、信息素养</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：原文说明正式法律文件中已经出现大量 AI 生成内容。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：它暗示 AI 内容已经进入制度文件，不只是私人聊天。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义、搭配题、翻译题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：contain 与 document/report/complaint 搭配多译“包含”；与 disease/inflation 搭配多译“遏制”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：include, hold / exclude, omit&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The report contained AI-generated text that no editor had checked. 译：报告包含未经编辑核查的 AI 生成文本。 2. A public notice should contain clear information about citizens' rights. 译：公共通知应包含关于公民权利的清晰信息。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Educational policies should contain clear rules for AI-generated text. 译：教育政策应包含关于 AI 生成文本的明确规则。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育诚信、公共政策、科技治理</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -344,17 +344,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>flag non-existent cases</t>
+          <t>As well as inventing cases, ...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Canadian courts have flagged non-existent cases in 79 rulings so far this year. 译：截至今年目前，加拿大法院已经在 79 份裁决中标出了并不存在的案例。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：标出不存在的案例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：flag 作动词是“标出、提示、警示”；non-existent 是高频否定形容词。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：flag 原为“旗帜”，动词表示“打标记”；non-existent = non- 不 + existent 存在的。English: to flag a problem is to draw attention to it as requiring notice or action.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：case 在本文是“案例/判例”；non-existent cases 指被引用但现实中不存在的判例。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical, evidential, institutional</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：As well as inventing cases, AI chatbots often encourage people to litigate, urge them not to settle and overstate their chances of winning. 译：AI 聊天机器人不仅会编造案例，还经常鼓励人们提起诉讼，劝他们不要和解，并夸大他们胜诉的可能性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：不仅会编造案例，还……&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：句首 `As well as + doing` 后接主句，常引出附加危害或附加好处。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：as well as = 除……之外也；inventing cases 是动名词短语。English: this structure adds one action before listing the main actions of the subject.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：invent 不只指“发明”，也可指“编造”，如 invent an excuse/story/case。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, cumulative, critical</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：这一数据证明 AI 幻觉已经影响法院裁决。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题可能问加拿大法院发现了什么；flag 可被替换为 identify, mark, point out。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Editors flagged non-existent sources before the report was released. 译：编辑在报告发布前标出了不存在的来源。 2. The database flagged non-existent addresses in the application forms. 译：数据库标出了申请表中不存在的地址。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public institutions should flag non-existent sources before misinformation spreads. 译：公共机构应在错误信息扩散前标出不存在的来源。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：信息核验、学术诚信、公共治理</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用该结构把 AI 的危害从“编造案例”扩展到“助长诉讼、拒绝和解、夸大胜算”。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：结构本身体现递进：问题不止一个，而且后果更广。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长难句、并列谓语、段落逻辑题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：先抓主语 AI chatbots，再看三个并列动词 encourage/urge/overstate。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：besides doing, in addition to doing / instead of doing&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. As well as saving time, AI tools can reduce costs and widen access to basic services. 译：AI 工具除了节省时间，还能降低成本并扩大基础服务的可及性。 2. As well as spreading rumours, social media can deepen anger and weaken trust. 译：社交媒体除了传播谣言，还会加深愤怒并削弱信任。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：As well as improving efficiency, technology should protect fairness and accountability. 译：科技除了提高效率，还应保护公平和问责。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：长难句仿写、科技利弊、社会责任</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -366,17 +366,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>false citations</t>
+          <t>a grievance</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Most false citations have been made by people representing themselves. 译：大多数虚假引用都是由自行代理的当事人提交的。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：虚假引用。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：citation 可指论文引用，也可指法律判例引用；false 是事实错误，不只是“不真诚”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：cite = 引用，citation = 引文/引用项；false = 虚假的、不正确的。English: in legal writing, a citation points to authority; a false citation points to a source that is wrong or fabricated.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：citation 还可指交通罚单；在学术/法律语境中是“引用”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：negative, academic/legal integrity</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A grievance that would have been a few sentences is now more like ten to 12 pages. 译：原本只有几句话的申诉，现在更像是十到十二页的长篇材料。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：委屈、抱怨、申诉。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：grievance 比 complaint 更正式，常用于劳动、校园、制度不公语境。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：grieve = 悲伤/感到不公，grievance = 因不公而提出的抱怨或申诉。English: a grievance is a complaint about unfair treatment, often in a workplace or institution.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：complaint 可指抱怨或起诉状；grievance 更强调受到不公待遇后的正式申诉。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, institutional, sometimes emotional</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：虚假引用暴露了 AI 输出未核验带来的诚信和程序风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译中不要译为“错误引证”过轻，应体现“虚假/捏造”风险。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The journal rejected the paper after reviewers found several false citations. 译：审稿人发现数处虚假引用后，期刊拒绝了这篇论文。 2. False citations can destroy public trust in legal and academic documents. 译：虚假引用会破坏公众对法律和学术文件的信任。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：False citations should be treated as a serious threat to academic integrity. 译：虚假引用应被视为对学术诚信的严重威胁。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：学术诚信、法律诚信、信息素养</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 把本来简短的申诉扩写成冗长材料，增加法院和对方负担。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能用 complaint, objection, resentment 替换。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The worker filed a grievance after being denied equal pay. 译：这名员工在被拒绝同工同酬后提出申诉。 2. A school should handle every grievance fairly and quickly. 译：学校应公平、快速地处理每一项申诉。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Institutions should create fair channels through which citizens can raise a grievance. 译：机构应建立公平渠道，让公民能够提出申诉。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场生活、教育公平、公共伦理</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -388,17 +388,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>encourage people to litigate</t>
+          <t>overstate their chances of winning</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI chatbots often encourage people to litigate. 译：AI 聊天机器人经常鼓励人们提起诉讼。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：鼓励人们打官司。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：litigate 是正式法律动词，比 sue 更偏“进行诉讼程序”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：encourage sb to do = 鼓励某人做某事；litigate = 提起/进行诉讼。English: litigate refers to pursuing a dispute through the court process.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：encourage 在负面语境中可译为“助长”，不一定是褒义“鼓励”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical in context</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI chatbots often overstate their chances of winning. 译：AI 聊天机器人经常夸大他们胜诉的可能性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：夸大他们赢的机会。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：over- 前缀表示“过度”；attitude 题中 overstate 常体现批评。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：overstate = over- 过度 + state 陈述；chance = 可能性。English: to overstate a risk, benefit or chance is to present it as greater than it really is.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：state 作动词是“陈述”，不是“国家”；chance 可指机会，也可指概率。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical, cautionary</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 不只是提供文字，还改变人的决策，可能增加无谓诉讼。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题中 encourage 若与 risky behaviour 搭配，可能带负面含义。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Poor legal advice may encourage people to litigate instead of negotiating. 译：糟糕的法律建议可能鼓励人们诉讼，而不是谈判。 2. A responsible platform should not encourage people to litigate without checking the facts. 译：负责任的平台不应在未核查事实的情况下鼓励人们诉讼。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Technology should solve disputes, not encourage people to litigate unnecessarily. 译：科技应解决争端，而不是鼓励人们进行不必要的诉讼。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：公共治理、社会责任、平台责任</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 输出让当事人误判案件胜算，从而增加诉讼。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换包括 exaggerate, inflate；反义陷阱是 understate。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The advertisement overstated the product's chances of improving sleep. 译：广告夸大了该产品改善睡眠的可能性。 2. Investors lost money because the start-up overstated its chances of success. 译：投资者亏钱是因为这家初创公司夸大了成功可能性。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Media platforms should not overstate the chances of quick success through technology. 译：媒体平台不应夸大通过科技快速成功的可能性。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技宣传、健康产品、创业经济</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -410,17 +410,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>urge someone not to settle</t>
+          <t>embolden litigants to bring discrimination claims</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI chatbots often urge people not to settle and overstate their chances of winning. 译：AI 聊天机器人经常劝人不要和解，并夸大他们胜诉的可能性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：敦促某人不要和解。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：settle 在法律语境中是“和解”，不是“定居”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：urge sb to do = 催促/力劝某人做；settle = 解决争端/达成和解。English: settle can mean to resolve a dispute without continuing a trial.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：settle: 1. 定居；2. 安顿；3. 解决；4. 和解。本文取法律和解义。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：cautionary, negative in context</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Chatbots embolden litigants to bring discrimination claims. 译：聊天机器人会给诉讼当事人壮胆，让他们提出歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：使诉讼当事人更大胆地提出歧视索赔。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：embolden = 使更有胆量，常带“壮胆后采取更激进行动”的意味。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：em- 使成为 + bold 大胆；claim = 主张/索赔。English: embolden someone to do something means to give them confidence, sometimes excessive confidence, to act.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：claim: 1. 声称；2. 主张；3. 索赔；4. 权利要求。本文是法律索赔/主张。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical, legal, behaviour-focused</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 可能让当事人更激进，拒绝本来更理性的和解。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：完形中 settle 与 litigate、dispute、claim 搭配时优先译为“和解/解决”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The chatbot urged the tenant not to settle, even though the offer was fair. 译：聊天机器人劝租客不要和解，尽管对方提议是公平的。 2. A mediator helps both sides settle before costs become too high. 译：调解员帮助双方在成本过高前达成和解。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public platforms should encourage people to settle reasonable disputes, not intensify conflict. 译：公共平台应鼓励人们解决合理争端，而不是加剧冲突。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：冲突解决、公共伦理、职场纠纷</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 让当事人更敢提出歧视索赔，但这些主张未必有充分依据。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：attitude 题中 embolden 可能暗示作者担心行为被助长。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Anonymous forums may embolden users to make extreme accusations. 译：匿名论坛可能让用户更大胆地提出极端指控。 2. Clear evidence can embolden workers to bring discrimination claims against unfair employers. 译：清晰证据能让员工更有底气向不公平雇主提出歧视索赔。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Digital tools should empower citizens, but they should not embolden people to bring discrimination claims without evidence. 译：数字工具应赋能公民，但不应让人们在没有证据的情况下大胆提出歧视索赔。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场公平、平台责任、社会正义</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -432,17 +432,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>overstate their chances of winning</t>
+          <t>litigate</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI chatbots often overstate their chances of winning. 译：AI 聊天机器人经常夸大他们胜诉的可能性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：夸大他们赢的机会。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：over- 前缀表示“过度”；attitude 题中 overstate 常体现批评。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：overstate = over- 过度 + state 陈述；chance = 可能性。English: to overstate a risk, benefit or chance is to present it as greater than it really is.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：state 作动词是“陈述”，不是“国家”；chance 可指机会，也可指概率。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical, cautionary</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：AI chatbots often encourage people to litigate, urge them not to settle and overstate their chances of winning. 译：AI 聊天机器人经常鼓励人们提起诉讼，劝他们不要和解，并夸大他们胜诉的可能性。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：提起诉讼；进行诉讼。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：正式法律动词，比 sue 更强调通过法院程序解决争端。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：litigate = 通过诉讼处理争端；litigation = 诉讼。English: litigate means to take a dispute through legal proceedings.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：sue 更强调“起诉某人”；litigate 更强调“进行诉讼过程”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 输出让当事人误判案件胜算，从而增加诉讼。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换包括 exaggerate, inflate；反义陷阱是 understate。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The advertisement overstated the product's chances of improving sleep. 译：广告夸大了该产品改善睡眠的可能性。 2. Investors lost money because the start-up overstated its chances of success. 译：投资者亏钱是因为这家初创公司夸大了成功可能性。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Media platforms should not overstate the chances of quick success through technology. 译：媒体平台不应夸大通过科技快速成功的可能性。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技宣传、健康产品、创业经济</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 可能鼓励人们诉讼，而不是理性和解。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：该词暗示公共系统成本上升，因为诉讼会消耗法院资源。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义辨析、完形搭配、态度题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：litigate 和 settle 常形成反义关系：打官司 vs 和解。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：go to court, sue, bring a case / settle, negotiate&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The neighbours decided to litigate after mediation failed. 译：调解失败后，邻居决定提起诉讼。 2. Companies should not litigate every disagreement if negotiation can solve the problem. 译：如果谈判能解决问题，公司不应把每个分歧都诉诸法院。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：A mature society should help citizens resolve conflicts before they need to litigate. 译：成熟社会应帮助公民在需要诉讼之前解决冲突。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：公共治理、职场纠纷、社会责任</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -454,17 +454,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>embolden litigants to bring discrimination claims</t>
+          <t>barrister</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Chatbots embolden litigants to bring discrimination claims. 译：聊天机器人会给诉讼当事人壮胆，让他们提出歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：使诉讼当事人更大胆地提出歧视索赔。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：embolden = 使更有胆量，常带“壮胆后采取更激进行动”的意味。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：em- 使成为 + bold 大胆；claim = 主张/索赔。English: embolden someone to do something means to give them confidence, sometimes excessive confidence, to act.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：claim: 1. 声称；2. 主张；3. 索赔；4. 权利要求。本文是法律索赔/主张。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：critical, legal, behaviour-focused</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Antony Sendall, a British employment barrister, says chatbots embolden litigants to bring discrimination claims. 译：英国劳动就业领域的大律师 Antony Sendall 说，聊天机器人会给诉讼当事人壮胆，让他们提出歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：大律师；出庭律师。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：英美法律职业词。英国 barrister 通常指出庭辩护/陈述的律师，不等同于所有 lawyer。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：bar 与律师行业有关，barrister 是有资格在高等法院出庭的律师。English: a barrister is a lawyer, especially in Britain, who specialises in courtroom advocacy.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：lawyer 泛指律师；barrister 偏出庭；solicitor 偏咨询、文书和客户事务。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, professional, British legal term</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 让当事人更敢提出歧视索赔，但这些主张未必有充分依据。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：attitude 题中 embolden 可能暗示作者担心行为被助长。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Anonymous forums may embolden users to make extreme accusations. 译：匿名论坛可能让用户更大胆地提出极端指控。 2. Clear evidence can embolden workers to bring discrimination claims against unfair employers. 译：清晰证据能让员工更有底气向不公平雇主提出歧视索赔。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Digital tools should empower citizens, but they should not embolden people to bring discrimination claims without evidence. 译：数字工具应赋能公民，但不应让人们在没有证据的情况下大胆提出歧视索赔。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场公平、平台责任、社会正义</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章引用一位就业法大律师，增强论证可信度。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：用专业人士观点说明 AI 正在改变诉讼行为。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：背景知识、身份同位语、细节题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：遇到 `X, a barrister, says...`，逗号中间是身份同位语。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：courtroom lawyer, advocate / layperson, chatbot&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. A barrister argued the case after the AI platform prepared the documents. 译：AI 平台准备文件后，一名大律师出庭辩论该案。 2. The barrister warned that weak evidence could damage the claim. 译：这位大律师警告说，薄弱证据可能损害该索赔。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Even when digital tools handle paperwork, a barrister may still be needed for complex arguments. 译：即使数字工具处理文书，复杂论证仍可能需要大律师。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律职业、AI 与职业分工</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -476,17 +476,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>a grievance</t>
+          <t>correspondence</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A grievance that would have been a few sentences is now more like ten to 12 pages. 译：原本只有几句话的申诉，现在更像是十到十二页的长篇材料。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：委屈、抱怨、申诉。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：grievance 比 complaint 更正式，常用于劳动、校园、制度不公语境。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：grieve = 悲伤/感到不公，grievance = 因不公而提出的抱怨或申诉。English: a grievance is a complaint about unfair treatment, often in a workplace or institution.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：complaint 可指抱怨或起诉状；grievance 更强调受到不公待遇后的正式申诉。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, institutional, sometimes emotional</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：His clients receive correspondence and documents written by AI from opposing parties acting without lawyers. 译：他的客户会收到未聘请律师的对方当事人发来的由 AI 撰写的信件和文件。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：通信；往来信件；函件。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：正式书面词，常用于商务、法律、行政场景。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：correspond = 通信/相一致；correspondence = 通信、信件往来。English: correspondence refers to letters or emails exchanged between people or organisations.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：还可指“对应关系”，如 correspondence between theory and reality。本文是“往来信件”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, administrative/legal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 把本来简短的申诉扩写成冗长材料，增加法院和对方负担。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能用 complaint, objection, resentment 替换。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The worker filed a grievance after being denied equal pay. 译：这名员工在被拒绝同工同酬后提出申诉。 2. A school should handle every grievance fairly and quickly. 译：学校应公平、快速地处理每一项申诉。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Institutions should create fair channels through which citizens can raise a grievance. 译：机构应建立公平渠道，让公民能够提出申诉。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场生活、教育公平、公共伦理</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 生成的法律函件已经进入当事人之间的正式往来。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：它说明 AI 影响的不只是法院文件，也影响诉讼双方沟通。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义、商务法律阅读。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：与 documents, receive, written by 搭配时多译“函件/通信”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：letters, emails, written communication / conversation, speech&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The lawyer reviewed all correspondence before replying to the claim. 译：律师在回复索赔前审查了所有往来函件。 2. Schools should keep clear correspondence with parents during a crisis. 译：学校在危机期间应与家长保持清晰的书面沟通。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Transparent correspondence between institutions and citizens can reduce misunderstanding. 译：机构与公民之间透明的书面沟通可以减少误解。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：商务沟通、公共治理、教育管理</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -498,17 +498,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>self-representing litigants</t>
+          <t>improperly</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In cases with self-representing litigants in America, the number of documents filed in the first 180 days is 158% higher than in the pre-AI era. 译：在美国自行代理当事人的案件中，前 180 天提交的文件数量比 AI 出现前高出 158%。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：自行代理的诉讼当事人。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：复合形容词 self-representing 修饰 litigants，表示“没有律师代理”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：self- = 自己；represent = 代理；litigant = 诉讼当事人。English: the compound adjective compresses a full relative clause: litigants who represent themselves.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：self- 前缀常见：self-control 自控，self-reliance 自立，self-employed 自雇。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A student was ordered to pay the University of Ottawa C$10,000, partly for using AI improperly to prepare her legal challenge. 译：一名学生被判向渥太华大学支付 10,000 加元，部分原因是她不当使用 AI 来准备法律挑战。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：不适当地；不正当地；违规地。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：improperly 是责任判断副词，说明问题不在“使用 AI”本身，而在“不当使用”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：improper = 不合适的/不正当的；-ly 变副词。English: improperly means in a way that breaks rules, standards or proper procedure.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：properly/improperly 常用于程序、方法和规范判断。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：negative, procedural, evaluative</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：数据显示 AI 让自行代理案件的文件数量暴增。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长难句翻译中要把 `with self-representing litigants` 译成“有自行代理当事人的案件”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Self-representing litigants often need forms written in plain English. 译：自行代理的诉讼当事人常需要用简明英语写成的表格。 2. Courts face heavier workloads when self-representing litigants submit excessive documents. 译：自行代理当事人提交过多文件时，法院工作负担会加重。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public institutions should support self-representing litigants without lowering standards of evidence. 译：公共机构应支持自行代理的诉讼当事人，但不能降低证据标准。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律援助、社会公平、公共服务</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：学生被罚的原因之一是使用 AI 的方式不符合规则。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：作者借此区分“谨慎使用 AI”与“不当依赖 AI”。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题、原因题、翻译题。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：注意 improperly 的范围：修饰 using AI，不是修饰 prepare 本身。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：inappropriately, wrongly, against rules / properly, appropriately&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The clinic was criticised for using patient data improperly. 译：这家诊所因不当使用患者数据而受到批评。 2. A student who uses AI improperly may violate academic rules. 译：不当使用 AI 的学生可能违反学术规则。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI should not be banned simply because some people use it improperly. 译：不能仅因为有些人不当使用 AI 就彻底禁止它。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育诚信、科技治理、医疗伦理</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -520,17 +520,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>in the pre-AI era</t>
+          <t>sue someone in a federal court</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：The number of documents filed in the first 180 days is 158% higher than in the pre-AI era. 译：案件开始后前 180 天提交的文件数量比 AI 出现前高出 158%。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在 AI 出现前的时代。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：pre- 前缀表示“之前”，常用于时间对比和历史分期。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：pre- = before，era = 时代。English: pre-AI, pre-pandemic and pre-industrial are compact ways to mark a before-and-after contrast.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：era 指“时代、时期”，常与 technological, digital, post-war 搭配。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：analytical, periodising</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In March Nippon Life, an insurer, sued OpenAI in a federal court in Chicago. 译：今年 3 月，保险公司 Nippon Life 在芝加哥联邦法院起诉 OpenAI。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在联邦法院起诉某人/某机构。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：sue 是法律高频基础动词，比 litigate 更具体地表示“起诉”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：sue + sb = 起诉某人；in a court = 在某法院。English: to sue someone is to start a legal case against them, usually seeking a remedy or damages.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：sue for damages = 起诉索赔；sue over privacy/pollution/contracts = 因隐私/污染/合同问题起诉。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, formal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者通过 AI 前后数据对比说明法院文件数量增长。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：图表/数据题中 pre- 与 post- 是时间对照信号。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. In the pre-AI era, students spent more time searching for basic information. 译：在 AI 出现前，学生花更多时间查找基础信息。 2. The company's workflow was slower in the pre-AI era. 译：在 AI 出现前，这家公司的工作流程更慢。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：In the pre-AI era, access to expert knowledge was far less equal than it is today. 译：在 AI 出现前，人们获得专家知识的机会远没有今天平等。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技变化、教育学习、职场效率</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：Nippon Life 起诉 OpenAI，把 AI 责任问题推向平台层面。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：起诉对象从个人转为 AI 公司，文章讨论范围扩大。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题、法律动作识别。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：sue 不等于 accuse；sue 是启动诉讼，accuse 是提出指控。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：bring a lawsuit against, take someone to court / settle with, drop a case&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Consumers sued the company in a federal court after a data leak. 译：数据泄露后，消费者在联邦法院起诉该公司。 2. The city sued the factory over years of illegal pollution. 译：该市因多年非法污染起诉这家工厂。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Citizens should be able to sue powerful organisations when their rights are violated. 译：当权利受到侵犯时，公民应能够起诉强势组织。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律公平、消费者保护、环境保护&lt;br&gt;&lt;b&gt;归一化合并&lt;/b&gt;：用户词表 sued 归一化为 sue someone in a federal court。</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -542,17 +542,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>opposing parties acting without lawyers</t>
+          <t>insurer</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：His clients receive correspondence and documents written by AI from opposing parties acting without lawyers. 译：他的客户会收到未聘请律师的对方当事人发来的由 AI 撰写的信件和文件。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：没有律师代理的对方当事人。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：opposing party 是法律/谈判中的“对方”；acting without lawyers 是现在分词后置定语。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：opposing = 对立的，party = 一方/当事人；act without = 在没有……情况下行动。English: party in legal English means a person or organisation involved in a case, not a celebration or political party.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：party: 政党/聚会/一方当事人；correspondence: 通信/往来信件。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：In March Nippon Life, an insurer, sued OpenAI in a federal court in Chicago. 译：今年 3 月，保险公司 Nippon Life 在芝加哥联邦法院起诉 OpenAI。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：保险公司；承保人。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：经济/商业阅读基础词，来自 insure；不要和 ensure 混淆。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：insure = 给……投保/承保；insurer = 保险公司；insured = 被保险人。English: an insurer is a company that provides insurance and bears certain financial risks.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：insure 投保/承保；ensure 确保；assure 使确信。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：business, financial, neutral</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 让没有律师的一方也能制造大量正式文件。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时别把 party 译成“派对”；要译为“当事方”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Opposing parties acting without lawyers may misunderstand court rules. 译：没有律师代理的对方当事人可能误解法院规则。 2. The mediator helped opposing parties acting without lawyers reach a settlement. 译：调解员帮助没有律师代理的对立双方达成和解。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Public systems should offer clear guidance to opposing parties acting without lawyers. 译：公共系统应为没有律师代理的对立当事方提供清晰指引。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律公平、公共服务、冲突解决</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：Nippon Life 作为保险公司起诉 OpenAI，说明 AI 法律风险已经进入商业责任领域。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：保险公司通常重视风险定价，因此它起诉 AI 公司具有商业风险意味。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：形近词辨析、商业阅读、同位语识别。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：看到 `Nippon Life, an insurer,`，逗号内是同位语解释公司身份。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：insurance company, underwriter / customer, insured person&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The insurer refused to pay because the claim lacked evidence. 译：保险公司因索赔缺乏证据而拒绝赔付。 2. An insurer must price risk carefully when new technologies appear. 译：新技术出现时，保险公司必须谨慎评估风险定价。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：An insurer can encourage safer behaviour by rewarding companies that reduce risk. 译：保险公司可以通过奖励降低风险的企业来鼓励更安全的行为。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：经济生活、商业风险、科技责任</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -564,17 +564,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>relying on AI can prove expensive</t>
+          <t>allege that</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：And relying on AI can prove expensive. 译：依赖 AI 也可能代价高昂。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：依赖 AI 可能最终证明很昂贵。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：prove + adj. = 结果证明是；expensive 可指金钱或代价。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：rely on = 依赖；prove expensive = 结果代价高昂。English: prove followed by an adjective describes the outcome, not the act of giving evidence.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：prove 不只表示“证明”，也可表示“结果是”；expensive 可引申为“造成严重后果”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：warning, concise, evaluative</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Nippon Life sued OpenAI, alleging that ChatGPT had enabled an ex-employee to make what it says is a meritless discrimination claim. 译：Nippon Life 起诉 OpenAI，声称 ChatGPT 帮助一名前雇员提出了一项其所称毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：声称；指称；宣称某事发生。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：新闻法律报道高频词，表示“提出说法但尚未被证实”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：allege + that 从句 = 声称……；allegation = 指控/说法。English: allege attributes a claim to a party without confirming it as fact.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：alleged = 被指称的/所谓的；注意不是 confirmed。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, cautious, attribution-focused</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：该句开启一组因 AI 使用不当而被罚款或道歉的例子。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题不要译成“证明昂贵”，应译为“结果可能代价高昂”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Relying on AI can prove expensive when legal facts are not checked. 译：如果不核查法律事实，依赖 AI 可能代价高昂。 2. Relying on cheap repairs can prove expensive when safety is ignored. 译：如果忽视安全，依赖廉价维修可能最终代价高昂。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Relying on AI can prove expensive when efficiency is pursued at the expense of responsibility. 译：当效率以牺牲责任为代价时，依赖 AI 可能代价高昂。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技依赖、健康建议、学习工具、职场效率</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用 alleging 把 Nippon Life 的说法与事实区分开。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：体现新闻写作的谨慎：报道主张，但不替法院下结论。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：事实/观点区分、态度题、法律报道。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：含 allege 的句子，答案选项不能把 allegation 当 confirmed fact。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：claim, assert, contend / prove, confirm&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Residents alleged that the factory had polluted the river for years. 译：居民声称该工厂多年来污染河流。 2. The report alleged that the platform had misled users about privacy. 译：报告声称该平台在隐私方面误导用户。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Before society accepts what a company alleges, evidence should be examined carefully. 译：在社会接受公司声称的内容之前，应仔细审查证据。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：新闻阅读、环境争议、科技责任</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -586,17 +586,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>legal challenge against removal from a programme</t>
+          <t>make what it says is a meritless discrimination claim</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：She used AI improperly to prepare her legal challenge against her removal from a PhD programme. 译：她不当使用 AI 来准备针对自己被博士项目除名的法律挑战。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：针对被项目除名提出法律挑战。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：challenge 作名词是“质疑/挑战”；removal from... 是“从……中除名/移除”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：legal challenge = 法律上的质疑；against = 针对；removal = 移除/免职/除名。English: removal can refer to dismissal from a post, exclusion from a programme, or taking something away.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：removal: 1. 移除；2. 免职；3. 搬迁；4. 除名。本文是教育项目中的除名。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, institutional</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：ChatGPT had enabled an ex-employee to make what it says is a meritless discrimination claim. 译：ChatGPT 帮助一名前雇员提出了一项 Nippon Life 所称毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：提出其所称毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：嵌套名词性从句 + 法律评价词。what it says is... 表示“它所称的……”，保留说法来源。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：make a claim = 提出主张/索赔；what it says is... = 它所称是……的东西；meritless = 无依据的。English: the clause avoids stating that the claim is truly meritless; it reports Nippon Life's view.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：claim 可指声称、主张、索赔；merit 在法律中指“实质依据”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, cautious, negative from Nippon Life's perspective</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：学生因在法律挑战中不当使用 AI 而被判支付费用。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：细节题会把 programme removal 改写为 being expelled/excluded from a doctoral programme。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The researcher filed a legal challenge against removal from the grant programme. 译：这名研究人员就自己被科研资助项目除名提出法律挑战。 2. A clear appeals process can reduce legal challenges against removal from school programmes. 译：清晰的申诉程序可以减少针对被学校项目除名的法律挑战。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Universities should explain removal from a programme clearly before students bring a legal challenge. 译：大学应在学生提出法律挑战之前，清楚解释项目除名决定。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：教育公平、程序正义、校园治理</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：保险公司认为 ChatGPT 促成了前员工提出无依据的歧视索赔。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：政治/责任意味在于：AI 公司是否要为用户拿模型输出去索赔负责。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长难句、嵌套从句、事实与观点区分。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：翻译时要把 what it says is 译出来，避免把“无依据”当作者或法院定论。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：make an unfounded claim, bring a baseless claim / make a well-founded claim&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The employee made what the company says is a meritless discrimination claim after using an online template. 译：这名员工使用在线模板后，提出了公司所称毫无根据的歧视索赔。 2. A court should examine evidence before treating a claim as meritless. 译：法院在认定主张毫无根据之前，应审查证据。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Digital tools should help citizens make valid claims, not make what opponents describe as meritless discrimination claims. 译：数字工具应帮助公民提出有效主张，而不是提出对方所称毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场公平、法律责任、长难句翻译</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -608,17 +608,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>be caught out</t>
+          <t>a hospitality firm</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Even lawyers have been caught out. 译：即使是律师也会中招。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：被抓到在外面；引申为“被发现出错、被难住、露馅”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语，out 表示暴露或出局。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：catch sb out = 发现某人错误/让某人措手不及；被动 be caught out = 被发现出错。English: the phrase often means to expose someone's mistake or lack of preparation.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：catch 不只是“抓住”，还可指“发现问题、让人措手不及”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：informal, slightly critical</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：She recovered 7,000 pounds in fees from a hospitality firm after engaging Garfield AI. 译：她在使用 Garfield AI 后，从一家酒店餐饮公司追回了 7,000 英镑费用。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：酒店餐饮公司； hospitality 行业企业。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：hospitality 不是“好客”这一抽象义时，常指酒店、餐饮、旅游接待行业。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：hospitality = 好客/接待服务业；firm = 公司。English: a hospitality firm is a business in hotels, restaurants, catering or related services.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：firm 可指“公司”，也可作形容词“坚定的”。hospitality 可指待客，也可指服务业。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：business, neutral</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者强调 AI 错误不仅困扰普通人，也会让专业律师出错。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时可译为“中招、被发现犯错、露馅”，按语境选择。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The firm was caught out by outdated safety rules. 译：这家公司因不了解过时的安全规则而中招。 2. Several students were caught out after submitting essays with fake sources. 译：几名学生提交含有虚假来源的论文后被发现。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：People are easily caught out when they trust convenient tools without checking the facts. 译：人们如果不核查事实就相信便利工具，很容易中招。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：学习诚信、职场风险、信息核验</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：这家公司是被追回费用的一方，用来展示 AI 法律工具的积极案例。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：行业词显示 AI 法律服务进入普通劳动/商业纠纷，而不只是高端法律市场。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义、商业场景词。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：hospitality 与 firm/industry/worker 搭配时，优先译为“酒店餐饮/接待服务业”。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：hotel-and-restaurant company, catering business / hospital, charity&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Workers at a hospitality firm complained about unpaid wages. 译：一家酒店餐饮公司的员工投诉工资未付。 2. A hospitality firm can lose customers quickly if service quality falls. 译：如果服务质量下降，酒店餐饮公司可能迅速失去顾客。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：A hospitality firm should respect workers' rights as much as customer satisfaction. 译：酒店餐饮公司应像重视顾客满意一样重视员工权利。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场权益、经济生活、服务业</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -630,17 +630,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AI hallucinations</t>
+          <t>do the documentary heavy lifting</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：A top New York firm apologised to a court for errors caused by AI hallucinations. 译：一家纽约顶级律所因 AI 幻觉造成的错误向法院道歉。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：AI 的幻觉；指 AI 编造看似真实但并不存在的信息。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：科技类核心术语，可用于理解 AI 可靠性和信息核验。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：hallucination 本义是“幻觉”，AI hallucination 是比喻用法，指模型生成虚假内容。English: in AI, hallucination means fluent but false output, not a human medical symptom.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：hallucination 在医学中是“幻觉”，在 AI 中是“编造性输出”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：technical, cautionary, negative</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Garfield's platform did the documentary heavy lifting. 译：Garfield 的平台完成了繁重的文书工作。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：完成繁重的文书工作。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：documentary 的熟词僻义 + heavy lifting 的比喻义；非常适合记成整块。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：documentary = 文件的/文书的，不是纪录片；heavy lifting = 重活/最费力部分。English: doing the documentary heavy lifting means handling the demanding paperwork.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：documentary: 纪录片/文书的；heavy lifting: 搬重物/艰巨任务。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：metaphorical, practical, slightly informal</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 幻觉导致律所向法院道歉，说明专业人士也不能免于风险。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：词义题可能问 hallucinations 在科技语境中的含义，应选 fabricated output，而非 mental illness。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. AI hallucinations can produce confident answers with false statistics. 译：AI 幻觉可能生成带有虚假统计数据却语气自信的答案。 2. Doctors should not rely on AI hallucinations when making clinical decisions. 译：医生做临床决策时不应依赖 AI 编造内容。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI hallucinations remind us that speed is meaningless without accuracy. 译：AI 幻觉提醒我们，没有准确性，速度毫无意义。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技生活、健康医疗、教育诚信</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 平台负责文书重活，人类大律师负责出庭辩论。&lt;br&gt;&lt;b&gt;暗示意思/政治意味/诙谐意味&lt;/b&gt;：暗示 AI 的合理位置是辅助繁重流程，而不是完全替代专业判断。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义、比喻理解、职业分工。&lt;br&gt;&lt;b&gt;答题技巧&lt;/b&gt;：不要把 documentary 译成“纪录片”；这里与 legal documents 呼应。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：handle the paperwork, do the hard administrative work / make final judgment&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. AI can do the documentary heavy lifting in routine contract review. 译：AI 可以在常规合同审查中完成繁重文书工作。 2. The software did the documentary heavy lifting, while the doctor checked the final report. 译：软件完成了繁重文书工作，而医生检查最终报告。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI should do the documentary heavy lifting, while humans retain responsibility for judgment and ethics. 译：AI 应完成繁重文书工作，而人类保留判断和伦理责任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：AI 与职业、医疗文书、教育行政、职场效率&lt;br&gt;&lt;b&gt;归一化合并&lt;/b&gt;：用户词表 do the documentary heavy lifting 与旧卡 documentary heavy lifting 合并。</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -652,17 +652,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>contractual dispute</t>
+          <t>citing fabricated cases</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Lawyers on both sides of a contractual dispute in Mississippi were fined for citing fabricated cases. 译：在密西西比州一起合同纠纷中，双方律师都因引用捏造案例而被罚款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：合同纠纷。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：contractual 是 contract 的形容词；dispute 是法律、国际关系、职场文章高频词。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：contract = 合同；-ual 形容词后缀；dispute = 争端/纠纷。English: contractual describes something arising from or governed by a contract.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：dispute 作名词是争端，作动词是质疑/争论；contract 作名词是合同，作动词可指收缩。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, legal, neutral</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Lawyers were fined for citing fabricated cases. 译：律师因引用捏造案例而被罚款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：引用捏造的案例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：cite 是学术和法律高频动词；fabricated 强调人为编造。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：cite = 引用；fabricate = 制造/编造；fabricated cases = 被捏造的案例。English: fabricated is stronger than false because it suggests deliberate creation of something untrue.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：fabricate 可指制造物品，也可指编造故事、证据、数据。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：negative, integrity-focused, legal</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：合同纠纷中的双方律师都引用捏造案例，说明 AI 错误影响专业法律实践。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：阅读中 dispute 可被替换为 conflict, disagreement, legal row。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The supplier and the factory entered a contractual dispute over delivery dates. 译：供应商和工厂因交货日期陷入合同纠纷。 2. Mediation can resolve a contractual dispute before it reaches court. 译：调解可以在合同纠纷进入法院前解决问题。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Clear rules can prevent a contractual dispute from damaging long-term cooperation. 译：清晰规则可以防止合同纠纷损害长期合作。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场商业、经济生活、法律阅读</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：捏造案例触碰法律职业底线，因此双方律师被罚。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换包括 quote invented precedents, rely on fake authorities。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The court punished the lawyer for citing fabricated cases in a brief. 译：法院因律师在诉状中引用捏造案例而处罚他。 2. A university may discipline students who cite fabricated cases or sources. 译：大学可能处分引用捏造案例或来源的学生。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：No society can build trust if professionals cite fabricated cases or data. 译：如果专业人士引用捏造案例或数据，社会就无法建立信任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：学术诚信、职业伦理、公共信任</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -674,262 +674,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cite fabricated cases</t>
+          <t>caught out</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Lawyers were fined for citing fabricated cases. 译：律师因引用捏造案例而被罚款。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：引用捏造的案例。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：cite 是学术和法律高频动词；fabricated 强调人为编造。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：cite = 引用；fabricate = 制造/编造；fabricated cases = 被捏造的案例。English: fabricated is stronger than false because it suggests deliberate creation of something untrue.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：fabricate 可指制造物品，也可指编造故事、证据、数据。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：negative, integrity-focused, legal</t>
+          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Even lawyers have been caught out. 译：即使是律师也会中招。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：被抓到在外面；引申为“被发现出错、被难住、露馅”。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：熟词短语，out 表示暴露或出局。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：catch sb out = 发现某人错误/让某人措手不及；被动 be caught out = 被发现出错。English: the phrase often means to expose someone's mistake or lack of preparation.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：catch 不只是“抓住”，还可指“发现问题、让人措手不及”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：informal, slightly critical</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：捏造案例触碰法律职业底线，因此双方律师被罚。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：同义替换包括 quote invented precedents, rely on fake authorities。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The court punished the lawyer for citing fabricated cases in a brief. 译：法院因律师在诉状中引用捏造案例而处罚他。 2. A university may discipline students who cite fabricated cases or sources. 译：大学可能处分引用捏造案例或来源的学生。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：No society can build trust if professionals cite fabricated cases or data. 译：如果专业人士引用捏造案例或数据，社会就无法建立信任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：学术诚信、职业伦理、公共信任</t>
+          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者强调 AI 错误不仅困扰普通人，也会让专业律师出错。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译时可译为“中招、被发现犯错、露馅”，按语境选择。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The firm was caught out by outdated safety rules. 译：这家公司因不了解过时的安全规则而中招。 2. Several students were caught out after submitting essays with fake sources. 译：几名学生提交含有虚假来源的论文后被发现。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：People are easily caught out when they trust convenient tools without checking the facts. 译：人们如果不核查事实就相信便利工具，很容易中招。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：学习诚信、职场风险、信息核验</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>bear responsibility for model inventions</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Some believe that AI labs should bear responsibility for their models' inventions. 译：有人认为，AI 实验室应当为其模型的“发明”承担责任。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：为模型的发明/编造内容承担责任。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：bear responsibility for 是作文和阅读中的责任表达，bear 不是“熊”，而是“承担”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：bear = 承担/承受；responsibility = 责任；for 引出责任对象。English: bear responsibility for is more formal than be responsible for and often appears in law, politics and ethics.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：bear: 1. 熊；2. 承受；3. 忍受；4. 生育。本文取“承担”。invention 在本文带讽刺，指模型编造出来的东西。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, ethical, legal; mildly ironic because inventions refers to fake outputs</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：责任讨论从用户错误转向 AI 公司是否应为模型输出负责。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：议论文主旨题常围绕 who should bear responsibility 展开。&lt;br&gt;&lt;b&gt;同义替换/错误选项信号&lt;/b&gt;：be liable for, be accountable for / escape responsibility, deny any role&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Platforms should bear responsibility for foreseeable harm caused by their products. 译：平台应为其产品造成的可预见伤害承担责任。 2. Parents and schools both bear responsibility for children's digital habits. 译：家长和学校都应为孩子的数字习惯承担责任。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Powerful technology companies should bear responsibility for model inventions that damage public trust. 译：强大的科技公司应为损害公共信任的模型编造内容承担责任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：社会责任、科技伦理、环境保护、教育治理</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>allege that</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Nippon Life sued OpenAI, alleging that ChatGPT had enabled an ex-employee to make a meritless discrimination claim. 译：Nippon Life 起诉 OpenAI，声称 ChatGPT 帮助一名前雇员提出一项毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：声称、指称。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：allege 是新闻和法律报道高频动词，表示“未经最终证实的指控”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：allege + that 从句 = 声称……；allegation = 指控/说法。English: allege signals that the writer is reporting a claim, not confirming it as fact.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：alleged 作形容词常译为“所谓的、被指称的”，保留未定事实状态。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, cautious, attribution-focused</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者用 alleging 避免把 Nippon Life 的说法直接当成事实。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度/事实题中 allege 提醒读者区分 claim 和 fact。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Residents alleged that the factory had polluted the river for years. 译：居民声称该工厂多年来污染河流。 2. The report alleged that the company had misled consumers about health benefits. 译：报告声称该公司在健康益处方面误导消费者。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Before the public accepts what a platform alleges, evidence should be carefully examined. 译：在公众接受平台所声称的内容之前，证据应被仔细审查。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：新闻阅读、法律报道、环境争议</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>enable someone to make a meritless claim</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：ChatGPT had enabled an ex-employee to make what Nippon Life says is a meritless discrimination claim. 译：ChatGPT 帮助一名前雇员提出了 Nippon Life 所称毫无根据的歧视索赔。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：使某人能够提出毫无根据的主张。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：enable sb to do 是因果结构；meritless 是法律高频负面词，表示“没有价值/没有依据”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：enable = 使能够；merit = 价值/优点/根据；-less = 没有。English: a meritless claim lacks legal or factual basis.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：merit 不只是“优点”，在法律中可指案件或主张的“实质依据”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, evaluative, negative</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Nippon Life 的诉讼逻辑是：AI 让前员工更容易提出无依据索赔。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：因果题可能把 enable 改写为 allow, make it possible for。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Poorly designed tools can enable users to make meritless claims with confidence. 译：设计不佳的工具会让用户自信地提出毫无根据的主张。 2. The court dismissed the meritless claim after reviewing the evidence. 译：法院审查证据后驳回了这项毫无根据的主张。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Technology should enable citizens to defend their rights, not enable them to make meritless claims. 译：科技应让公民能够维护权利，而不是让他们提出毫无根据的主张。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技伦理、法律公平、平台责任</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>punitive damages</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Nippon is seeking $10m in punitive damages. 译：Nippon Life 正在寻求 1,000 万美元的惩罚性赔偿。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：惩罚性的损害赔偿。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：punitive 与 punish 同源；damages 复数在法律中指“赔偿金”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：punitive = 惩罚性的；damages = 法律赔偿金。English: punitive damages are intended to punish wrongdoing, not only compensate loss.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：damage 不可数常指损害；damages 复数是法律赔偿金。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal, financial, severe</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：该金额显示 AI 责任问题可能产生巨大法律和经济后果。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题中 damages 要译为“赔偿金”，不是“损害”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The company faced punitive damages after hiding safety risks from consumers. 译：该公司因向消费者隐瞒安全风险而面临惩罚性赔偿。 2. Punitive damages can deter firms from ignoring public welfare. 译：惩罚性赔偿可以阻止企业忽视公共福祉。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Punitive damages may be necessary when companies repeatedly put profit before safety. 译：当企业反复把利润置于安全之前时，惩罚性赔偿可能是必要的。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：消费者保护、企业责任、经济法律阅读</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>insist that ChatGPT is not a lawyer</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：OpenAI insists that ChatGPT is "not a lawyer". 译：OpenAI 坚称 ChatGPT “不是律师”。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：坚称 ChatGPT 不是律师。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：insist that 在新闻语境中常表示“坚称某事实”，不是“坚持要求”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：insist = 坚持说/坚称；that 从句说明坚持的内容。English: insist can report a firm claim, especially when a party rejects responsibility.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：insist on doing = 坚持做；insist that + 陈述句 = 坚称。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：defensive, legal, corporate</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：OpenAI 用该句划清产品与专业法律服务之间的责任边界。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：态度题可据此判断 OpenAI 是否承认责任：它是在否认或限制责任。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The platform insists that its health chatbot is not a doctor. 译：该平台坚称其健康聊天机器人不是医生。 2. The company insisted that the software was only a tool, not a substitute for experts. 译：该公司坚称这款软件只是工具，而不是专家的替代品。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Companies may insist that AI is only a tool, but they still need to reduce foreseeable risks. 译：企业可以坚称 AI 只是工具，但仍需要减少可预见风险。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技责任、企业声明、健康与法律 AI</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>used with caution</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Used with caution, AI can be beneficial. 译：谨慎使用时，AI 可以带来好处。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在谨慎使用的情况下。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：过去分词短语作条件状语；作文高频平衡句型。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：caution = 谨慎；used with caution = if it is used carefully。English: the past participle phrase compresses a conditional clause and makes the sentence concise.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：caution 可作名词“谨慎/警告”，也可作动词“警告”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：balanced, prudent, formal</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：作者在批评风险后承认 AI 的正面价值，形成平衡结论。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：篇章题中该句是转折/让步后的平衡点。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Used with caution, online medical information can help patients ask better questions. 译：谨慎使用时，网上医疗信息能帮助患者提出更好的问题。 2. Used with caution, generative AI can reduce routine paperwork in schools. 译：谨慎使用时，生成式 AI 可以减少学校中的日常文书工作。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Used with caution, technology can improve efficiency without weakening human responsibility. 译：谨慎使用时，科技可以提高效率而不削弱人的责任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技创新、健康信息、教育学习、职场效率</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>recover fees from a firm</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Tamires Camal Taquidir recovered 7,000 pounds in fees from a hospitality firm after engaging Garfield AI. 译：Tamires Camal Taquidir 在使用 Garfield AI 后，从一家酒店餐饮公司追回了 7,000 英镑费用。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：从一家公司追回费用。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：recover 在法律/金融语境中是“追回、收回”，不是“康复”。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：recover = 恢复/追回；fees = 费用；from 引出付款方。English: recover money means to get back money owed or lost.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：recover: 1. 康复；2. 恢复；3. 追回金钱；4. 找回。本文取追回费用。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：legal/financial, positive outcome</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：这是 AI 有益的一面：帮助用户完成文书并追回费用。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义题可能把 recover 错译为“康复”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The workers recovered unpaid wages from the factory after filing a complaint. 译：工人投诉后从工厂追回了拖欠工资。 2. Consumers used a legal service to recover fees from the airline. 译：消费者使用法律服务从航空公司追回费用。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Simple legal tools can help ordinary people recover fees from powerful institutions. 译：简单法律工具可以帮助普通人从强势机构追回费用。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：消费者保护、职场权益、法律援助</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>AI-powered law firm approved by regulators</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Garfield AI calls itself the world's first AI-powered law firm approved by regulators. 译：Garfield AI 自称是世界上第一家获得监管机构批准的 AI 驱动律师事务所。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：由 AI 驱动并获监管机构批准的律师事务所。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：AI-powered 是复合形容词；approved by regulators 是后置定语，监管合规是科技治理主题。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：powered by = 由……驱动；regulator = 监管机构；approved by = 获……批准。English: AI-powered describes a service whose main operation relies on AI technology.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：power 在 powered by 中不是“权力”，而是“驱动、提供动力”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：promotional but institutionally cautious</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Garfield AI 代表较正规、受监管的 AI 法律服务，与随意使用聊天机器人形成对比。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：长难句翻译中两个后置修饰要层层前置。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. An AI-powered clinic approved by regulators must still protect patient privacy. 译：获监管机构批准的 AI 驱动诊所仍必须保护患者隐私。 2. AI-powered learning tools approved by regulators can help schools reduce routine work. 译：获监管机构批准的 AI 驱动学习工具能帮助学校减少日常工作。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI-powered services approved by regulators can expand access while maintaining public trust. 译：获监管机构批准的 AI 驱动服务可以扩大可及性，同时维护公共信任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：科技治理、健康服务、教育技术、职业转型</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>documentary heavy lifting</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Garfield's platform did the documentary heavy lifting. 译：Garfield 的平台完成了繁重的文书工作。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：完成文书方面的重活。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：heavy lifting 是比喻，指最费力、最核心或最繁重的工作；documentary 在此指文件/文书相关。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：documentary 不只是“纪录片”，也可作形容词“文件的、文书的”；heavy lifting = 重体力活，引申为艰巨任务。English: the phrase suggests AI handled the tedious paperwork rather than courtroom advocacy.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：documentary: 1. 纪录片；2. 文件的/文书的。heavy lifting: 体力重活/艰巨任务。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：metaphorical, practical, slightly informal</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 的价值在于处理文书重活，但出庭辩论仍由人类律师完成。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：熟词僻义题可能把 documentary 错看成“纪录片”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The software did the documentary heavy lifting, while the doctor made the final decision. 译：软件完成了繁重的文书工作，而医生作出最终决定。 2. AI can do the documentary heavy lifting in routine contract review. 译：AI 可以在常规合同审查中完成繁重文书工作。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：AI should do the documentary heavy lifting, while humans retain responsibility for judgment and ethics. 译：AI 应完成繁重文书工作，而人类保留判断和伦理责任。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：职场效率、AI 分工、医疗文书、教育行政</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>argue the case in court</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：Dominic Li, a barrister, argued the case in court. 译：大律师 Dominic Li 在法庭上为该案进行辩论。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：在法庭上辩论这个案件。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：argue 在法律和学术语境中是“论证、辩护”，不是普通吵架。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：argue = 争论/论证/辩护；case = 案件/论点。English: to argue a case means to present legal reasons before a court.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：argue 可指吵架，也可指“提出论证”；case 可指案件，也可指“论点、理由”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：formal, professional, legal</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：AI 处理文书，人类律师负责法庭辩论，体现人机分工。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：翻译题要按法律语境译为“为案件辩论/陈述理由”。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. The lawyer argued the case in court after AI helped organise the documents. 译：AI 帮助整理文件后，律师在法庭上为案件辩论。 2. A scientist must argue the case for environmental protection with clear evidence. 译：科学家必须用清晰证据论证环境保护的理由。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：Citizens can argue the case for public responsibility only when facts are carefully checked. 译：只有在事实被仔细核查后，公民才能论证公共责任的重要性。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：法律、议论文、环境保护、公共政策</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>human lawyers still have their place</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;原文/拓展表达&lt;/b&gt;：For now, human lawyers still have their place. 译：至少目前，人类律师仍有其不可替代的位置。&lt;br&gt;&lt;b&gt;字面含义&lt;/b&gt;：人类律师仍有自己的位置。&lt;br&gt;&lt;b&gt;考研核心考点&lt;/b&gt;：have one's place = 仍有价值/仍有适用场景；用于平衡论证。&lt;br&gt;&lt;b&gt;词汇拆解&lt;/b&gt;：中文：place 不只是地点，也可指角色、位置、价值。English: to have one's place means to remain useful or appropriate within a changing system.&lt;br&gt;&lt;b&gt;熟词辟义/一词多义&lt;/b&gt;：place: 地方/位置/角色/社会地位。本文是“角色和价值”。&lt;br&gt;&lt;b&gt;语气色彩&lt;/b&gt;：balanced, concluding, pragmatic</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：文章承认 AI 有用，但结论强调专业人类判断仍不可替代。&lt;br&gt;&lt;b&gt;特殊考查方式&lt;/b&gt;：主旨题和态度题可据此判断作者不是简单反 AI，而是主张谨慎分工。&lt;br&gt;&lt;b&gt;多场景例句&lt;/b&gt;：1. Even in an age of online courses, human teachers still have their place. 译：即使在在线课程时代，人类教师仍有其价值。 2. Automated tools are useful, but human editors still have their place. 译：自动化工具很有用，但人类编辑仍有其位置。&lt;br&gt;&lt;b&gt;作文应用&lt;/b&gt;：In the age of artificial intelligence, human judgment still has its place in education and public life. 译：在人工智能时代，人的判断在教育和公共生活中仍有其价值。&lt;br&gt;&lt;b&gt;其他可用地方&lt;/b&gt;：AI 与职业、教育学习、医疗健康、文化传承</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
         <is>
           <t>外刊精读</t>
         </is>

</xml_diff>